<commit_message>
[양대용] 랜덤 스테이지 선택형 던전 기반 데이터 테이블 구성(Dungeon, Stage, StageGroup, MapData, MonsterSpawn, DropObject, StateReward)
</commit_message>
<xml_diff>
--- a/Shared/XLS/Character.xlsx
+++ b/Shared/XLS/Character.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="136">
   <si>
     <t>!Enum</t>
     <phoneticPr fontId="10" type="noConversion"/>
@@ -630,6 +630,18 @@
   </si>
   <si>
     <t>Knight</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>LevelStepDesc</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>!string</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">범위+{1}, 데미지+{2}, </t>
     <phoneticPr fontId="9" type="noConversion"/>
   </si>
 </sst>
@@ -3914,18 +3926,18 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J29"/>
+  <dimension ref="A1:K29"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9" style="9"/>
     <col min="2" max="3" width="9" style="2"/>
     <col min="4" max="4" width="21.75" style="2" customWidth="1"/>
-    <col min="5" max="5" width="62.375" style="2" customWidth="1"/>
-    <col min="6" max="10" width="32" style="2" bestFit="1" customWidth="1"/>
-    <col min="11" max="16384" width="9" style="2"/>
+    <col min="5" max="6" width="62.375" style="2" customWidth="1"/>
+    <col min="7" max="11" width="32" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" s="7" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -3933,7 +3945,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="8"/>
       <c r="B2" s="5" t="s">
         <v>3</v>
@@ -3947,23 +3959,26 @@
       <c r="E2" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="11" t="s">
+        <v>133</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="I2" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="J2" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="K2" s="2" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="8"/>
       <c r="B3" s="11" t="s">
         <v>7</v>
@@ -3977,11 +3992,11 @@
       <c r="E3" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="11" t="s">
+        <v>134</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>92</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>86</v>
       </c>
       <c r="H3" s="2" t="s">
         <v>86</v>
@@ -3992,8 +4007,11 @@
       <c r="J3" s="2" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K3" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B4" s="2">
         <v>1001</v>
       </c>
@@ -4006,23 +4024,26 @@
       <c r="E4" s="18" t="s">
         <v>107</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="18" t="s">
+        <v>135</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="H4" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="I4" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="I4" s="2" t="s">
+      <c r="J4" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="J4" s="2" t="s">
+      <c r="K4" s="2" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B5" s="2">
         <v>1002</v>
       </c>
@@ -4035,23 +4056,23 @@
       <c r="E5" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="G5" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="H5" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="H5" s="2" t="s">
+      <c r="I5" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="I5" s="2" t="s">
+      <c r="J5" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="J5" s="2" t="s">
+      <c r="K5" s="2" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B6" s="2">
         <v>1003</v>
       </c>
@@ -4064,23 +4085,23 @@
       <c r="E6" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="G6" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="H6" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="H6" s="2" t="s">
+      <c r="I6" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="I6" s="2" t="s">
+      <c r="J6" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="J6" s="2" t="s">
+      <c r="K6" s="2" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B7" s="2">
         <v>1004</v>
       </c>
@@ -4093,23 +4114,23 @@
       <c r="E7" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="G7" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="H7" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="H7" s="2" t="s">
+      <c r="I7" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="I7" s="2" t="s">
+      <c r="J7" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="J7" s="2" t="s">
+      <c r="K7" s="2" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B8" s="2">
         <v>1005</v>
       </c>
@@ -4122,36 +4143,41 @@
       <c r="E8" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="G8" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="G8" s="2" t="s">
+      <c r="H8" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="H8" s="2" t="s">
+      <c r="I8" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="I8" s="2" t="s">
+      <c r="J8" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="J8" s="2" t="s">
+      <c r="K8" s="2" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="E9" s="18"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="F9" s="18"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="E14" s="18"/>
-    </row>
-    <row r="19" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="F14" s="18"/>
+    </row>
+    <row r="19" spans="5:6" x14ac:dyDescent="0.3">
       <c r="E19" s="18"/>
-    </row>
-    <row r="24" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="F19" s="18"/>
+    </row>
+    <row r="24" spans="5:6" x14ac:dyDescent="0.3">
       <c r="E24" s="18"/>
-    </row>
-    <row r="29" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="F24" s="18"/>
+    </row>
+    <row r="29" spans="5:6" x14ac:dyDescent="0.3">
       <c r="E29" s="18"/>
+      <c r="F29" s="18"/>
     </row>
   </sheetData>
   <phoneticPr fontId="9" type="noConversion"/>

</xml_diff>